<commit_message>
genes more than 49 variants
</commit_message>
<xml_diff>
--- a/Outputs_primates/AllGenes_Potential_CPDs.xlsx
+++ b/Outputs_primates/AllGenes_Potential_CPDs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uofh-my.sharepoint.com/personal/miadesin_cougarnet_uh_edu/Documents/Documents/Ricardo_lab/GitHub/kondrashov/Outputs_primates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="156" documentId="13_ncr:1_{8A2AFB6C-B6BE-D242-8FA1-EF65A1680E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBD0D20B-0FCC-4C18-8F22-AD19154620D6}"/>
+  <xr:revisionPtr revIDLastSave="205" documentId="13_ncr:1_{8A2AFB6C-B6BE-D242-8FA1-EF65A1680E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4D3ACBE-0207-4BDC-BC90-25D80907F3D5}"/>
   <bookViews>
-    <workbookView xWindow="7416" yWindow="0" windowWidth="15720" windowHeight="12336" xr2:uid="{BC6F7999-E049-F441-AF63-5F5D062E3B8F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC6F7999-E049-F441-AF63-5F5D062E3B8F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="268">
   <si>
     <t>gene</t>
   </si>
@@ -815,20 +815,41 @@
     <t>NP_055610.1</t>
   </si>
   <si>
-    <t>orthologs</t>
-  </si>
-  <si>
     <t>Aln</t>
   </si>
   <si>
     <t>species</t>
+  </si>
+  <si>
+    <t>Unlike other CPDs, the human species only has the 'wild', all other species have the 'mut'      lollll!</t>
+  </si>
+  <si>
+    <t>Hannah's</t>
+  </si>
+  <si>
+    <t>at site 491</t>
+  </si>
+  <si>
+    <t>Nil</t>
+  </si>
+  <si>
+    <t>Looks like a CPD, except that flanking region contains one gap, but gap is consistent across alignment</t>
+  </si>
+  <si>
+    <t>This is valid, although Hannah did not detect it among her 2 CPDs. Maybe I filter the alignment to exclude the gaps?</t>
+  </si>
+  <si>
+    <t>valid CPD</t>
+  </si>
+  <si>
+    <t>Hannah detected 5 CPDs! LDLR Alignment should be filtered; there are multiple gaps in-between</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -852,25 +873,46 @@
     </font>
     <font>
       <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="7"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
       <color rgb="FF00B0F0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="7"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -900,16 +942,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1269,7 +1315,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>3</v>
@@ -1281,10 +1327,10 @@
         <v>5</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -1312,9 +1358,6 @@
       <c r="H2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="1">
-        <v>34</v>
-      </c>
       <c r="J2" s="3"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -2097,7 +2140,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>64</v>
       </c>
@@ -2123,33 +2166,36 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="5">
         <v>969</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="5">
         <v>1102</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G34" s="1" t="s">
+      <c r="G34" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="H34" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>67</v>
       </c>
@@ -2175,33 +2221,33 @@
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
+    <row r="36" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="D36" s="5">
+      <c r="D36" s="4">
         <v>438</v>
       </c>
-      <c r="E36" s="5">
+      <c r="E36" s="4">
         <v>475</v>
       </c>
-      <c r="F36" s="5" t="s">
+      <c r="F36" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G36" s="5" t="s">
+      <c r="G36" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H36" s="5" t="s">
+      <c r="H36" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>73</v>
       </c>
@@ -2227,7 +2273,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>73</v>
       </c>
@@ -2253,7 +2299,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>76</v>
       </c>
@@ -2279,7 +2325,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>76</v>
       </c>
@@ -2305,7 +2351,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>79</v>
       </c>
@@ -2331,33 +2377,33 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="5">
         <v>13</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42" s="5">
         <v>128</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="G42" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H42" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>81</v>
       </c>
@@ -2383,7 +2429,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>85</v>
       </c>
@@ -2409,7 +2455,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>87</v>
       </c>
@@ -2435,7 +2481,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>87</v>
       </c>
@@ -2461,7 +2507,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="47" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>90</v>
       </c>
@@ -2487,7 +2533,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>92</v>
       </c>
@@ -2666,81 +2712,81 @@
         <v>56</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
+    <row r="55" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D55" s="1">
+      <c r="D55" s="5">
         <v>2038</v>
       </c>
-      <c r="E55" s="1">
+      <c r="E55" s="5">
         <v>2055</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="F55" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="G55" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="H55" s="5" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+    <row r="56" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="5">
         <v>2157</v>
       </c>
-      <c r="E56" s="1">
+      <c r="E56" s="5">
         <v>2174</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="F56" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="G56" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="H56" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
+    <row r="57" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="D57" s="1">
+      <c r="D57" s="5">
         <v>75</v>
       </c>
-      <c r="E57" s="1">
+      <c r="E57" s="5">
         <v>75</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F57" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="G57" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="H57" s="5" t="s">
         <v>61</v>
       </c>
     </row>
@@ -2923,7 +2969,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>121</v>
       </c>
@@ -2949,7 +2995,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>121</v>
       </c>
@@ -2975,189 +3021,198 @@
         <v>124</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A67" s="1" t="s">
+    <row r="67" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C67" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="9">
         <v>223</v>
       </c>
-      <c r="E67" s="1">
+      <c r="E67" s="9">
         <v>249</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="F67" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="G67" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H67" s="1" t="s">
+      <c r="H67" s="9" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
+      <c r="I67" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="J67" s="9" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="7">
         <v>502</v>
       </c>
-      <c r="E68" s="1">
+      <c r="E68" s="7">
         <v>506</v>
       </c>
-      <c r="F68" s="1" t="s">
+      <c r="F68" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G68" s="1" t="s">
+      <c r="G68" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="H68" s="1" t="s">
+      <c r="H68" s="7" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="5" t="s">
+      <c r="J68" s="7" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C69" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="D69" s="5">
+      <c r="D69" s="6">
         <v>535</v>
       </c>
-      <c r="E69" s="5">
+      <c r="E69" s="6">
         <v>539</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F69" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G69" s="5" t="s">
+      <c r="G69" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H69" s="5" t="s">
+      <c r="H69" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
+    <row r="70" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C70" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="5">
         <v>227</v>
       </c>
-      <c r="E70" s="1">
+      <c r="E70" s="5">
         <v>229</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="F70" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="G70" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H70" s="1" t="s">
+      <c r="H70" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
+    <row r="71" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="5">
         <v>351</v>
       </c>
-      <c r="E71" s="1">
+      <c r="E71" s="5">
         <v>353</v>
       </c>
-      <c r="F71" s="1" t="s">
+      <c r="F71" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G71" s="1" t="s">
+      <c r="G71" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H71" s="1" t="s">
+      <c r="H71" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
+    <row r="72" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C72" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="5">
         <v>350</v>
       </c>
-      <c r="E72" s="1">
+      <c r="E72" s="5">
         <v>352</v>
       </c>
-      <c r="F72" s="1" t="s">
+      <c r="F72" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G72" s="1" t="s">
+      <c r="G72" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H72" s="1" t="s">
+      <c r="H72" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A73" s="1" t="s">
+    <row r="73" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C73" s="1" t="s">
+      <c r="C73" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="5">
         <v>416</v>
       </c>
-      <c r="E73" s="1">
+      <c r="E73" s="5">
         <v>419</v>
       </c>
-      <c r="F73" s="1" t="s">
+      <c r="F73" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="G73" s="1" t="s">
+      <c r="G73" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H73" s="1" t="s">
+      <c r="H73" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>128</v>
       </c>
@@ -3183,7 +3238,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>128</v>
       </c>
@@ -3209,33 +3264,33 @@
         <v>42</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A76" s="1" t="s">
+    <row r="76" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C76" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="5">
         <v>351</v>
       </c>
-      <c r="E76" s="1">
+      <c r="E76" s="5">
         <v>353</v>
       </c>
-      <c r="F76" s="1" t="s">
+      <c r="F76" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G76" s="1" t="s">
+      <c r="G76" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H76" s="1" t="s">
+      <c r="H76" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="77" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>128</v>
       </c>
@@ -3261,7 +3316,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>130</v>
       </c>
@@ -3287,7 +3342,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="79" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>130</v>
       </c>
@@ -3313,7 +3368,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>133</v>
       </c>
@@ -3339,7 +3394,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>135</v>
       </c>
@@ -3365,7 +3420,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>137</v>
       </c>
@@ -3391,7 +3446,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="83" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>137</v>
       </c>
@@ -3417,7 +3472,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="84" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>137</v>
       </c>
@@ -3443,7 +3498,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="85" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>137</v>
       </c>
@@ -3469,7 +3524,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="86" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>137</v>
       </c>
@@ -3495,7 +3550,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="87" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>144</v>
       </c>
@@ -3520,8 +3575,11 @@
       <c r="H87" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="J87" s="10" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>144</v>
       </c>
@@ -3547,7 +3605,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="89" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>144</v>
       </c>
@@ -3573,33 +3631,36 @@
         <v>42</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A90" s="1" t="s">
+    <row r="90" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B90" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C90" s="1" t="s">
+      <c r="C90" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="6">
         <v>88</v>
       </c>
-      <c r="E90" s="1">
+      <c r="E90" s="6">
         <v>125</v>
       </c>
-      <c r="F90" s="1" t="s">
+      <c r="F90" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G90" s="1" t="s">
+      <c r="G90" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H90" s="1" t="s">
+      <c r="H90" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="I90" s="6" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>144</v>
       </c>
@@ -3625,7 +3686,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="92" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>147</v>
       </c>
@@ -3651,7 +3712,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>147</v>
       </c>
@@ -3677,7 +3738,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="94" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>147</v>
       </c>
@@ -3703,7 +3764,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>152</v>
       </c>
@@ -3729,7 +3790,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>152</v>
       </c>
@@ -3807,55 +3868,55 @@
         <v>132</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A99" s="1" t="s">
+    <row r="99" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B99" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C99" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="5">
         <v>176</v>
       </c>
-      <c r="E99" s="1">
+      <c r="E99" s="5">
         <v>197</v>
       </c>
-      <c r="F99" s="1" t="s">
+      <c r="F99" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G99" s="1" t="s">
+      <c r="G99" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H99" s="1" t="s">
+      <c r="H99" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A100" s="1" t="s">
+    <row r="100" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C100" s="1" t="s">
+      <c r="C100" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="5">
         <v>413</v>
       </c>
-      <c r="E100" s="1">
+      <c r="E100" s="5">
         <v>434</v>
       </c>
-      <c r="F100" s="1" t="s">
+      <c r="F100" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G100" s="1" t="s">
+      <c r="G100" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H100" s="1" t="s">
+      <c r="H100" s="5" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4171,137 +4232,137 @@
         <v>186</v>
       </c>
     </row>
-    <row r="113" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="5" t="s">
+    <row r="113" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="B113" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="C113" s="5" t="s">
+      <c r="C113" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="D113" s="5">
+      <c r="D113" s="6">
         <v>142</v>
       </c>
-      <c r="E113" s="5">
+      <c r="E113" s="6">
         <v>142</v>
       </c>
-      <c r="F113" s="5" t="s">
+      <c r="F113" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G113" s="5" t="s">
+      <c r="G113" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H113" s="5" t="s">
+      <c r="H113" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A114" s="1" t="s">
+    <row r="114" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B114" s="1" t="s">
+      <c r="B114" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C114" s="1" t="s">
+      <c r="C114" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="5">
         <v>127</v>
       </c>
-      <c r="E114" s="1">
+      <c r="E114" s="5">
         <v>127</v>
       </c>
-      <c r="F114" s="1" t="s">
+      <c r="F114" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="G114" s="1" t="s">
+      <c r="G114" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H114" s="1" t="s">
+      <c r="H114" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A115" s="1" t="s">
+    <row r="115" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="B115" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C115" s="1" t="s">
+      <c r="C115" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="5">
         <v>82</v>
       </c>
-      <c r="E115" s="1">
+      <c r="E115" s="5">
         <v>82</v>
       </c>
-      <c r="F115" s="1" t="s">
+      <c r="F115" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="G115" s="1" t="s">
+      <c r="G115" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H115" s="1" t="s">
+      <c r="H115" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A116" s="1" t="s">
+    <row r="116" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B116" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C116" s="1" t="s">
+      <c r="C116" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="5">
         <v>77</v>
       </c>
-      <c r="E116" s="1">
+      <c r="E116" s="5">
         <v>77</v>
       </c>
-      <c r="F116" s="1" t="s">
+      <c r="F116" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="G116" s="1" t="s">
+      <c r="G116" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H116" s="1" t="s">
+      <c r="H116" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A117" s="1" t="s">
+    <row r="117" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B117" s="1" t="s">
+      <c r="B117" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C117" s="1" t="s">
+      <c r="C117" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="5">
         <v>126</v>
       </c>
-      <c r="E117" s="1">
+      <c r="E117" s="5">
         <v>126</v>
       </c>
-      <c r="F117" s="1" t="s">
+      <c r="F117" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G117" s="1" t="s">
+      <c r="G117" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="H117" s="1" t="s">
+      <c r="H117" s="5" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>189</v>
       </c>
@@ -4327,7 +4388,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="119" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>191</v>
       </c>
@@ -4353,7 +4414,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="120" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
         <v>191</v>
       </c>
@@ -4379,7 +4440,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="121" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A121" s="4" t="s">
         <v>191</v>
       </c>
@@ -4405,7 +4466,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>191</v>
       </c>
@@ -4431,7 +4492,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="123" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A123" s="4" t="s">
         <v>191</v>
       </c>
@@ -4457,7 +4518,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="124" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
         <v>191</v>
       </c>
@@ -4483,7 +4544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="125" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
         <v>193</v>
       </c>
@@ -4509,33 +4570,36 @@
         <v>22</v>
       </c>
     </row>
-    <row r="126" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="6" t="s">
+    <row r="126" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B126" s="6" t="s">
+      <c r="B126" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="C126" s="6" t="s">
+      <c r="C126" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="D126" s="6">
+      <c r="D126" s="8">
         <v>341</v>
       </c>
-      <c r="E126" s="6">
+      <c r="E126" s="8">
         <v>523</v>
       </c>
-      <c r="F126" s="6" t="s">
+      <c r="F126" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G126" s="6" t="s">
+      <c r="G126" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="H126" s="6" t="s">
+      <c r="H126" s="8" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J126" s="8" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>197</v>
       </c>

</xml_diff>